<commit_message>
Sites do William (16/10): Mais Seguranca 1107/1114, regras PFF2/sapato/54%, nova montagem
Coleta da Mais Seguranca (GO): 1107 R$ 78,00 e 1114 R$ 1,00, com leitor proprio (site em JavaScript). 1114: TR e Astro reprovados (pacote). Aderencia: 1114 aceita respirador/mascara PFF2; sapato = calcado; 1107 aceita tenis/bota/botina de seguranca; 1001 aceita 54%. normalizar_url mantem a rota '#/'. Montagem 2026-10-16_072850 (1107, 1113 e 1114 mudam). 62 testes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>

Claude-Session: https://claude.ai/code/session_019igg4Dt3whcevpShV6u178
</commit_message>
<xml_diff>
--- a/FNDE/Centro Oeste/Entrega/EPI UNIFORME/fnde_resultado_merge.xlsx
+++ b/FNDE/Centro Oeste/Entrega/EPI UNIFORME/fnde_resultado_merge.xlsx
@@ -1191,46 +1191,44 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Multiseg Comercio de Equipamentos de Seguranca Ltda</t>
+          <t>Mais Segurança EPI</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>10.498.304/0001-84</t>
+          <t>43.903.641/0001-69</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>https://www.multiseg.com.br/4458/tenis-de-segurana-antiderrapante-sticky-shoe-copa-branco-ca-44589</t>
+          <t>https://maisseguranca.online/#/produto-detalhes/nUNEWOBUivWtuxf5g7uS3ulpNCn2/-N4ce5UWWtjnB32sQoGd</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Tênis de Segurança Sticky Shoe Copa Branco Ca 44589 Antiderrapante</t>
+          <t>SAPATO IMPERMEAVEL ANTIDERRAPANTE PRETO MAN 41 - STICKY SHOES CA.39674</t>
         </is>
       </c>
       <c r="J12" s="6" t="n">
-        <v>89.59999999999999</v>
+        <v>78</v>
       </c>
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n"/>
       <c r="M12" s="6" t="n">
-        <v>89.59999999999999</v>
-      </c>
-      <c r="N12" s="6" t="n">
-        <v>32.85</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="N12" s="2" t="n"/>
       <c r="O12" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: Pac R$ 32,85 De 9 A 10 dia(s) Úteis</t>
+          <t>Frete não calculado (GO para GO)</t>
         </is>
       </c>
       <c r="P12" s="2" t="n"/>
@@ -1253,39 +1251,49 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>A MASTER ARTIGOS PARA PROTECAO INDIVIDUAL E INDUSTRIAL LTDA (A Master EPI)</t>
+          <t>Multiseg Comercio de Equipamentos de Seguranca Ltda</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>16.603.654/0001-40</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="3" t="n"/>
-      <c r="J13" s="2" t="n"/>
+          <t>10.498.304/0001-84</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>https://www.multiseg.com.br/4458/tenis-de-segurana-antiderrapante-sticky-shoe-copa-branco-ca-44589</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Tênis de Segurança Sticky Shoe Copa Branco Ca 44589 Antiderrapante</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>89.59999999999999</v>
+      </c>
       <c r="K13" s="2" t="n"/>
       <c r="L13" s="2" t="n"/>
-      <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="n"/>
+      <c r="M13" s="6" t="n">
+        <v>89.59999999999999</v>
+      </c>
+      <c r="N13" s="6" t="n">
+        <v>32.85</v>
+      </c>
       <c r="O13" s="3" t="inlineStr">
         <is>
-          <t>Preço não exibido (motivo não identificado)</t>
-        </is>
-      </c>
-      <c r="P13" s="5" t="inlineStr">
-        <is>
-          <t>https://www.amasterepi.com.br/busca?q=Cal%C3%A7ado%20De%20Seguran%C3%A7a%20Antiderrapante</t>
-        </is>
-      </c>
+          <t>Opção mais barata para o CEP 74933-130: Pac R$ 32,85 De 9 A 10 dia(s) Úteis</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1295,17 +1303,17 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>1108</t>
+          <t>1107</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>BOTA DE PVC/BORRACHA - IMPERMEÁVEL, SOLADO ANTIDERRAPANTE, CANO MÉDIO OU LONGO.</t>
+          <t>CALÇADO DE SEGURANÇA ANTIDERRAPANTE - PROTEÇÃO CONTRA AGENTES MECÂNICOS; IMPERMEÁVEL QUANDO APLICÁVEL.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E14" s="4" t="n">
@@ -1313,45 +1321,31 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>LOJAS 360 INDUSTRIA, COMERCIO, IMPORTACAO, EXPORTACAO LTDA</t>
+          <t>A MASTER ARTIGOS PARA PROTECAO INDIVIDUAL E INDUSTRIAL LTDA (A Master EPI)</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>27.061.442/0002-85</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t>https://www.lojas360.com.br/bicodepvc/bota-de-pvc-cano-longo-preta-com-forro-biqueira-composite?variant_id=5711</t>
-        </is>
-      </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>Bota de Pvc Cano Longo Preta Com Forro Biqueira Composite</t>
-        </is>
-      </c>
-      <c r="J14" s="6" t="n">
-        <v>176.61</v>
-      </c>
+          <t>16.603.654/0001-40</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="3" t="n"/>
+      <c r="J14" s="2" t="n"/>
       <c r="K14" s="2" t="n"/>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>PVC aceito como impermeável (equivalência).</t>
-        </is>
-      </c>
-      <c r="M14" s="6" t="n">
-        <v>176.61</v>
-      </c>
-      <c r="N14" s="6" t="n">
-        <v>1687.82</v>
-      </c>
+      <c r="L14" s="2" t="n"/>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2" t="n"/>
       <c r="O14" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: Frete Valor Prazo de Entrega e Observações: Logística Própria FAVORITA R$ 1.687,82 Até 5 a 6 dia(s) úteis após o faturamento do pedido FRETE GRÁTIS PA</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="n"/>
+          <t>Preço não exibido (motivo não identificado)</t>
+        </is>
+      </c>
+      <c r="P14" s="5" t="inlineStr">
+        <is>
+          <t>https://www.amasterepi.com.br/busca?q=Cal%C3%A7ado%20De%20Seguran%C3%A7a%20Antiderrapante</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1379,42 +1373,42 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>SEGURANCA TOTAL EPIS LTDA</t>
+          <t>LOJAS 360 INDUSTRIA, COMERCIO, IMPORTACAO, EXPORTACAO LTDA</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>39.268.527/0001-37</t>
+          <t>27.061.442/0002-85</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>https://www.segurancatotal.com.br/bota-pvc-impermeavel-branco</t>
+          <t>https://www.lojas360.com.br/bicodepvc/bota-de-pvc-cano-longo-preta-com-forro-biqueira-composite?variant_id=5711</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>Bota PVC Impermeável Innpro Cano Médio Branco CA 36025 (numeração innpro: 34/35)</t>
+          <t>Bota de Pvc Cano Longo Preta Com Forro Biqueira Composite</t>
         </is>
       </c>
       <c r="J15" s="6" t="n">
-        <v>55.05</v>
+        <v>176.61</v>
       </c>
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Característica não confirmada na página do produto: solado antiderrapante.</t>
+          <t>PVC aceito como impermeável (equivalência).</t>
         </is>
       </c>
       <c r="M15" s="6" t="n">
-        <v>55.05</v>
+        <v>176.61</v>
       </c>
       <c r="N15" s="6" t="n">
-        <v>18.4</v>
+        <v>1687.82</v>
       </c>
       <c r="O15" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: R$ 18,40 7 dias úteis PAC R$ 28,85 3 dias úteis SEDEX</t>
+          <t>Opção mais barata para o CEP 74933-130: Frete Valor Prazo de Entrega e Observações: Logística Própria FAVORITA R$ 1.687,82 Até 5 a 6 dia(s) úteis após o faturamento do pedido FRETE GRÁTIS PA</t>
         </is>
       </c>
       <c r="P15" s="2" t="n"/>
@@ -1437,7 +1431,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E16" s="4" t="n">
@@ -1445,40 +1439,42 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Casa do Pica-Pau Ltda</t>
+          <t>SEGURANCA TOTAL EPIS LTDA</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>50.223.823/0001-54</t>
+          <t>39.268.527/0001-37</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>https://www.casadopicapau.com.br/bota-galocha-baspan-ultraleve-pvc-cano-longo-azul-amarelo-nautica/p</t>
+          <t>https://www.segurancatotal.com.br/bota-pvc-impermeavel-branco</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>Bota Galocha Baspan Ultraleve de PVC Cano Longo</t>
+          <t>Bota PVC Impermeável Innpro Cano Médio Branco CA 36025 (numeração innpro: 34/35)</t>
         </is>
       </c>
       <c r="J16" s="6" t="n">
-        <v>60.41</v>
+        <v>55.05</v>
       </c>
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>PVC aceito como impermeável (equivalência).</t>
+          <t>Característica não confirmada na página do produto: solado antiderrapante.</t>
         </is>
       </c>
       <c r="M16" s="6" t="n">
-        <v>60.41</v>
-      </c>
-      <c r="N16" s="2" t="n"/>
+        <v>55.05</v>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>18.4</v>
+      </c>
       <c r="O16" s="3" t="inlineStr">
         <is>
-          <t>Frete não calculado (GO para GO) | frete real: R$ 18,70</t>
+          <t>Opção mais barata para o CEP 74933-130: R$ 18,40 7 dias úteis PAC R$ 28,85 3 dias úteis SEDEX</t>
         </is>
       </c>
       <c r="P16" s="2" t="n"/>
@@ -1501,7 +1497,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="E17" s="4" t="n">
@@ -1509,26 +1505,26 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>SINGULAR COMERCIO DE EQUIPAMENTOS DE PROTECAO INDIVIDUAL LTDA (Loja do EPI)</t>
+          <t>Casa do Pica-Pau Ltda</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>20.838.307/0001-73</t>
+          <t>50.223.823/0001-54</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>https://www.lojadoepi.com.br/bota-de-pvc-work-cano-medio-cor-preta-comprimento-28-cm-ca-36025-innpro-p3301?pp=/40.1438/</t>
+          <t>https://www.casadopicapau.com.br/bota-galocha-baspan-ultraleve-pvc-cano-longo-azul-amarelo-nautica/p</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>Bota de PVC Work Cano Médio Cor Preta Comprimento 28 cm CA 36025 INNPRO</t>
+          <t>Bota Galocha Baspan Ultraleve de PVC Cano Longo</t>
         </is>
       </c>
       <c r="J17" s="6" t="n">
-        <v>44.56</v>
+        <v>60.41</v>
       </c>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="inlineStr">
@@ -1537,14 +1533,12 @@
         </is>
       </c>
       <c r="M17" s="6" t="n">
-        <v>44.56</v>
-      </c>
-      <c r="N17" s="6" t="n">
-        <v>25.47</v>
-      </c>
+        <v>60.41</v>
+      </c>
+      <c r="N17" s="2" t="n"/>
       <c r="O17" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: Pac R$ 25,47 7 dia(s) útil(eis)</t>
+          <t>Frete não calculado (GO para GO) | frete real: R$ 18,70</t>
         </is>
       </c>
       <c r="P17" s="2" t="n"/>
@@ -1567,50 +1561,50 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>MS</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E18" s="4" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Panan</t>
+          <t>SINGULAR COMERCIO DE EQUIPAMENTOS DE PROTECAO INDIVIDUAL LTDA (Loja do EPI)</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>15.448.996/0001-70</t>
+          <t>20.838.307/0001-73</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>https://www.panan.com.br/pecas-e-epis/calcados/bota-pvc-cano-longo-n-41-bpcl11-vulcabras</t>
+          <t>https://www.lojadoepi.com.br/bota-de-pvc-work-cano-medio-cor-preta-comprimento-28-cm-ca-36025-innpro-p3301?pp=/40.1438/</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>Bota PVC Cano Longo N° 41 BPCL11 - Vulcabras</t>
+          <t>Bota de PVC Work Cano Médio Cor Preta Comprimento 28 cm CA 36025 INNPRO</t>
         </is>
       </c>
       <c r="J18" s="6" t="n">
-        <v>86.90000000000001</v>
+        <v>44.56</v>
       </c>
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>PVC aceito como impermeável (equivalência). Característica não confirmada na página do produto: solado antiderrapante.</t>
+          <t>PVC aceito como impermeável (equivalência).</t>
         </is>
       </c>
       <c r="M18" s="6" t="n">
-        <v>86.90000000000001</v>
+        <v>44.56</v>
       </c>
       <c r="N18" s="6" t="n">
-        <v>38.7</v>
+        <v>25.47</v>
       </c>
       <c r="O18" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: Correios Econômico R$ 38,70 7 a 9 dias úteis</t>
+          <t>Opção mais barata para o CEP 74933-130: Pac R$ 25,47 7 dia(s) útil(eis)</t>
         </is>
       </c>
       <c r="P18" s="2" t="n"/>
@@ -1623,56 +1617,60 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>1109</t>
+          <t>1108</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>LUVA DE PVC - CANO MÉDIO OU LONGO; PARA ATIVIDADES DE LIMPEZA.</t>
+          <t>BOTA DE PVC/BORRACHA - IMPERMEÁVEL, SOLADO ANTIDERRAPANTE, CANO MÉDIO OU LONGO.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>MS</t>
         </is>
       </c>
       <c r="E19" s="4" t="n">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>LOJAS 360 INDUSTRIA, COMERCIO, IMPORTACAO, EXPORTACAO LTDA</t>
+          <t>Panan</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>27.061.442/0002-85</t>
+          <t>15.448.996/0001-70</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>https://www.lojas360.com.br/luvas-de-seguranca/luva-de-pvc-sem-forro-palma-aspera-70cm-com-ombreira</t>
+          <t>https://www.panan.com.br/pecas-e-epis/calcados/bota-pvc-cano-longo-n-41-bpcl11-vulcabras</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>Luva de PVC Sem Forro Palma Áspera 70cm Com Ombreira</t>
+          <t>Bota PVC Cano Longo N° 41 BPCL11 - Vulcabras</t>
         </is>
       </c>
       <c r="J19" s="6" t="n">
-        <v>52.44</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="K19" s="2" t="n"/>
-      <c r="L19" s="2" t="n"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>PVC aceito como impermeável (equivalência). Característica não confirmada na página do produto: solado antiderrapante.</t>
+        </is>
+      </c>
       <c r="M19" s="6" t="n">
-        <v>52.44</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="N19" s="6" t="n">
-        <v>18.4</v>
+        <v>38.7</v>
       </c>
       <c r="O19" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: SEDEX R$ 28,85 Até 6 dias úteis após o faturamento do pedido.rn PAC R$ 18,40 Até 10 dias úteis após o faturamento do pedido.rn Logística Própria FAVOR</t>
+          <t>Opção mais barata para o CEP 74933-130: Correios Econômico R$ 38,70 7 a 9 dias úteis</t>
         </is>
       </c>
       <c r="P19" s="2" t="n"/>
@@ -1703,38 +1701,38 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>SINGULAR COMERCIO DE EQUIPAMENTOS DE PROTECAO INDIVIDUAL LTDA (Loja do EPI)</t>
+          <t>LOJAS 360 INDUSTRIA, COMERCIO, IMPORTACAO, EXPORTACAO LTDA</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>20.838.307/0001-73</t>
+          <t>27.061.442/0002-85</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>https://www.lojadoepi.com.br/luva-de-pvc-para-jatista-ca-43248-ldi-safety-107-p2283</t>
+          <t>https://www.lojas360.com.br/luvas-de-seguranca/luva-de-pvc-sem-forro-palma-aspera-70cm-com-ombreira</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>Luva de PVC para Jatista CA 43248 LDI Safety</t>
+          <t>Luva de PVC Sem Forro Palma Áspera 70cm Com Ombreira</t>
         </is>
       </c>
       <c r="J20" s="6" t="n">
-        <v>65.88</v>
+        <v>52.44</v>
       </c>
       <c r="K20" s="2" t="n"/>
       <c r="L20" s="2" t="n"/>
       <c r="M20" s="6" t="n">
-        <v>65.88</v>
+        <v>52.44</v>
       </c>
       <c r="N20" s="6" t="n">
-        <v>27.98</v>
+        <v>18.4</v>
       </c>
       <c r="O20" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: Pac R$ 27,98 7 dia(s) útil(eis)</t>
+          <t>Opção mais barata para o CEP 74933-130: SEDEX R$ 28,85 Até 6 dias úteis após o faturamento do pedido.rn PAC R$ 18,40 Até 10 dias úteis após o faturamento do pedido.rn Logística Própria FAVOR</t>
         </is>
       </c>
       <c r="P20" s="2" t="n"/>
@@ -1757,44 +1755,46 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E21" s="4" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Goiás Ferramentas</t>
+          <t>SINGULAR COMERCIO DE EQUIPAMENTOS DE PROTECAO INDIVIDUAL LTDA (Loja do EPI)</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>09.497.806/0001-01</t>
+          <t>20.838.307/0001-73</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>https://www.goiasferramentas.com.br/produto/615-luva-de-pvc-cano-longo-45cm-kalipso</t>
+          <t>https://www.lojadoepi.com.br/luva-de-pvc-para-jatista-ca-43248-ldi-safety-107-p2283</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>Luva de PVC Cano Longo 45cm Kalipso</t>
+          <t>Luva de PVC para Jatista CA 43248 LDI Safety</t>
         </is>
       </c>
       <c r="J21" s="6" t="n">
-        <v>23.33</v>
+        <v>65.88</v>
       </c>
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="n"/>
       <c r="M21" s="6" t="n">
-        <v>23.33</v>
-      </c>
-      <c r="N21" s="2" t="n"/>
+        <v>65.88</v>
+      </c>
+      <c r="N21" s="6" t="n">
+        <v>27.98</v>
+      </c>
       <c r="O21" s="3" t="inlineStr">
         <is>
-          <t>Frete não calculado (GO para GO)</t>
+          <t>Opção mais barata para o CEP 74933-130: Pac R$ 27,98 7 dia(s) útil(eis)</t>
         </is>
       </c>
       <c r="P21" s="2" t="n"/>
@@ -1821,35 +1821,35 @@
         </is>
       </c>
       <c r="E22" s="4" t="n">
-        <v>46306</v>
+        <v>46304</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Fermarcs Ferramentas</t>
+          <t>Goiás Ferramentas</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>08.615.223/0001-75</t>
+          <t>09.497.806/0001-01</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>https://www.fermarcsferramentas.com.br/luvas/luva-pvc-azul-s-forro-palma-lisa-35cm-ca34593</t>
+          <t>https://www.goiasferramentas.com.br/produto/615-luva-de-pvc-cano-longo-45cm-kalipso</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>Luva Pvc Azul S/ Forro Palma Lisa 35cm Ca34593</t>
+          <t>Luva de PVC Cano Longo 45cm Kalipso</t>
         </is>
       </c>
       <c r="J22" s="6" t="n">
-        <v>24.9</v>
+        <v>23.33</v>
       </c>
       <c r="K22" s="2" t="n"/>
       <c r="L22" s="2" t="n"/>
       <c r="M22" s="6" t="n">
-        <v>24.9</v>
+        <v>23.33</v>
       </c>
       <c r="N22" s="2" t="n"/>
       <c r="O22" s="3" t="inlineStr">
@@ -1867,60 +1867,54 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>1110</t>
+          <t>1109</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>LUVA DE LÁTEX FORRADA - CANO CURTO; TAMANHOS VARIADOS.</t>
+          <t>LUVA DE PVC - CANO MÉDIO OU LONGO; PARA ATIVIDADES DE LIMPEZA.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="E23" s="4" t="n">
-        <v>46308</v>
+        <v>46306</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>BHZ EPI DISTRIBUIDORA LTDA</t>
+          <t>Fermarcs Ferramentas</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>31.893.116/0001-20</t>
+          <t>08.615.223/0001-75</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>https://www.loja.bhzepi.com.br/luva-latex-amarela-forrada-ca-42023-imbat</t>
+          <t>https://www.fermarcsferramentas.com.br/luvas/luva-pvc-azul-s-forro-palma-lisa-35cm-ca34593</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>LUVA LATEX AMARELA FORRADA CA 42023 IMBAT (Tamanho: M)</t>
+          <t>Luva Pvc Azul S/ Forro Palma Lisa 35cm Ca34593</t>
         </is>
       </c>
       <c r="J23" s="6" t="n">
-        <v>5</v>
+        <v>24.9</v>
       </c>
       <c r="K23" s="2" t="n"/>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>Característica não confirmada na página do produto: cano curto.</t>
-        </is>
-      </c>
+      <c r="L23" s="2" t="n"/>
       <c r="M23" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="N23" s="6" t="n">
-        <v>20.62</v>
-      </c>
+        <v>24.9</v>
+      </c>
+      <c r="N23" s="2" t="n"/>
       <c r="O23" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: R$ 20,62 7 dias úteis PAC R$ 26,55 5 dias úteis Jadlog Package R$ 40,39 3 dias úteis SEDEX</t>
+          <t>Frete não calculado (GO para GO)</t>
         </is>
       </c>
       <c r="P23" s="2" t="n"/>
@@ -1943,7 +1937,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="E24" s="4" t="n">
@@ -1951,42 +1945,42 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>LOJAS 360 INDUSTRIA, COMERCIO, IMPORTACAO, EXPORTACAO LTDA</t>
+          <t>BHZ EPI DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>27.061.442/0002-85</t>
+          <t>31.893.116/0001-20</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>https://www.lojas360.com.br/luvas-de-seguranca/luva-latex-antiderrapante-orange-kalipso-c-a-32499?variant_id=4253</t>
+          <t>https://www.loja.bhzepi.com.br/luva-latex-amarela-forrada-ca-42023-imbat</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>Luva Látex Antiderrapante Orange Kalipso | C.A. 32499</t>
+          <t>LUVA LATEX AMARELA FORRADA CA 42023 IMBAT (Tamanho: M)</t>
         </is>
       </c>
       <c r="J24" s="6" t="n">
-        <v>12.26</v>
+        <v>5</v>
       </c>
       <c r="K24" s="2" t="n"/>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>Característica não confirmada na página do produto: forrada, cano curto.</t>
+          <t>Característica não confirmada na página do produto: cano curto.</t>
         </is>
       </c>
       <c r="M24" s="6" t="n">
-        <v>12.26</v>
+        <v>5</v>
       </c>
       <c r="N24" s="6" t="n">
-        <v>18.4</v>
+        <v>20.62</v>
       </c>
       <c r="O24" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: SEDEX R$ 28,85 Até 6 dias úteis após o faturamento do pedido.rn PAC R$ 18,40 Até 10 dias úteis após o faturamento do pedido.rn Logística Própria FAVOR</t>
+          <t>Opção mais barata para o CEP 74933-130: R$ 20,62 7 dias úteis PAC R$ 26,55 5 dias úteis Jadlog Package R$ 40,39 3 dias úteis SEDEX</t>
         </is>
       </c>
       <c r="P24" s="2" t="n"/>
@@ -2009,7 +2003,7 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E25" s="4" t="n">
@@ -2017,42 +2011,42 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>SUPRIFLEX SUPRIMENTOS ONLINE LTDA</t>
+          <t>LOJAS 360 INDUSTRIA, COMERCIO, IMPORTACAO, EXPORTACAO LTDA</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>46.412.993/0001-00</t>
+          <t>27.061.442/0002-85</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>https://www.supriflex.com.br/produto/luva-latex-multiuso-quality-forte-vabene-verde-p.html</t>
+          <t>https://www.lojas360.com.br/luvas-de-seguranca/luva-latex-antiderrapante-orange-kalipso-c-a-32499?variant_id=4253</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>Luva Látex Multiuso Quality Forte Vabene Verde P</t>
+          <t>Luva Látex Antiderrapante Orange Kalipso | C.A. 32499</t>
         </is>
       </c>
       <c r="J25" s="6" t="n">
-        <v>4.99</v>
+        <v>12.26</v>
       </c>
       <c r="K25" s="2" t="n"/>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>Característica não confirmada na página do produto: cano curto.</t>
+          <t>Característica não confirmada na página do produto: forrada, cano curto.</t>
         </is>
       </c>
       <c r="M25" s="6" t="n">
-        <v>4.99</v>
+        <v>12.26</v>
       </c>
       <c r="N25" s="6" t="n">
-        <v>28.06</v>
+        <v>18.4</v>
       </c>
       <c r="O25" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: R$ 28,06 11 dias úteis Correios - Mini Envios R$ 31,54 7 dias úteis Correios PAC R$ 32,18 7 dias úteis Jadlog - .Package</t>
+          <t>Opção mais barata para o CEP 74933-130: SEDEX R$ 28,85 Até 6 dias úteis após o faturamento do pedido.rn PAC R$ 18,40 Até 10 dias úteis após o faturamento do pedido.rn Logística Própria FAVOR</t>
         </is>
       </c>
       <c r="P25" s="2" t="n"/>
@@ -2075,36 +2069,34 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>14/10/2026</t>
-        </is>
+          <t>RS</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>46308</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>SEGURANCA TOTAL EPIS LTDA</t>
+          <t>SUPRIFLEX SUPRIMENTOS ONLINE LTDA</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>39.268.527/0001-37</t>
+          <t>46.412.993/0001-00</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>https://www.segurancatotal.com.br/luva-de-latex-kalipso-amarela-ca-13959</t>
+          <t>https://www.supriflex.com.br/produto/luva-latex-multiuso-quality-forte-vabene-verde-p.html</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>Luva de Látex Multiuso Kalipso Amarela CA13959 (Tamanho: P)</t>
+          <t>Luva Látex Multiuso Quality Forte Vabene Verde P</t>
         </is>
       </c>
       <c r="J26" s="6" t="n">
-        <v>4.69</v>
+        <v>4.99</v>
       </c>
       <c r="K26" s="2" t="n"/>
       <c r="L26" s="2" t="inlineStr">
@@ -2113,14 +2105,14 @@
         </is>
       </c>
       <c r="M26" s="6" t="n">
-        <v>4.69</v>
+        <v>4.99</v>
       </c>
       <c r="N26" s="6" t="n">
-        <v>18.4</v>
+        <v>28.06</v>
       </c>
       <c r="O26" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: R$ 18,40 7 dias úteis PAC</t>
+          <t>Opção mais barata para o CEP 74933-130: R$ 28,06 11 dias úteis Correios - Mini Envios R$ 31,54 7 dias úteis Correios PAC R$ 32,18 7 dias úteis Jadlog - .Package</t>
         </is>
       </c>
       <c r="P26" s="2" t="n"/>
@@ -2143,34 +2135,36 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="n">
-        <v>46304</v>
+          <t>SP</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Multiseg Comercio de Equipamentos de Seguranca Ltda</t>
+          <t>SEGURANCA TOTAL EPIS LTDA</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>10.498.304/0001-84</t>
+          <t>39.268.527/0001-37</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
-          <t>https://www.multiseg.com.br/1619/luva-ltex-neoprene-supermix-super-safety</t>
+          <t>https://www.segurancatotal.com.br/luva-de-latex-kalipso-amarela-ca-13959</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>Luva de Látex e Neoprene Super MIX Forrada Super Safety Bicolor - Ca 33333</t>
+          <t>Luva de Látex Multiuso Kalipso Amarela CA13959 (Tamanho: P)</t>
         </is>
       </c>
       <c r="J27" s="6" t="n">
-        <v>9.98</v>
+        <v>4.69</v>
       </c>
       <c r="K27" s="2" t="n"/>
       <c r="L27" s="2" t="inlineStr">
@@ -2179,14 +2173,14 @@
         </is>
       </c>
       <c r="M27" s="6" t="n">
-        <v>9.98</v>
+        <v>4.69</v>
       </c>
       <c r="N27" s="6" t="n">
-        <v>32.85</v>
+        <v>18.4</v>
       </c>
       <c r="O27" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: Pac R$ 32,85 De 9 A 10 dia(s) Úteis</t>
+          <t>Opção mais barata para o CEP 74933-130: R$ 18,40 7 dias úteis PAC</t>
         </is>
       </c>
       <c r="P27" s="2" t="n"/>
@@ -2199,56 +2193,60 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>1111</t>
+          <t>1110</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>LUVA DE NEOPRENE - TAMANHOS VARIADOS; PARA MANIPULAÇÃO COMPATÍVEL DE PRODUTOS QUÍMICOS.</t>
+          <t>LUVA DE LÁTEX FORRADA - CANO CURTO; TAMANHOS VARIADOS.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="E28" s="4" t="n">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>BHZ EPI DISTRIBUIDORA LTDA</t>
+          <t>Multiseg Comercio de Equipamentos de Seguranca Ltda</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>31.893.116/0001-20</t>
+          <t>10.498.304/0001-84</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>https://www.loja.bhzepi.com.br/luva-latex-neoprene-bicolor-ca16779-volk</t>
+          <t>https://www.multiseg.com.br/1619/luva-ltex-neoprene-supermix-super-safety</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>LUVA LATEX NEOPRENE BICOLOR CA16779 VOLK (Tamanho: M)</t>
+          <t>Luva de Látex e Neoprene Super MIX Forrada Super Safety Bicolor - Ca 33333</t>
         </is>
       </c>
       <c r="J28" s="6" t="n">
-        <v>13</v>
+        <v>9.98</v>
       </c>
       <c r="K28" s="2" t="n"/>
-      <c r="L28" s="2" t="n"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Característica não confirmada na página do produto: cano curto.</t>
+        </is>
+      </c>
       <c r="M28" s="6" t="n">
-        <v>13</v>
+        <v>9.98</v>
       </c>
       <c r="N28" s="6" t="n">
-        <v>20.62</v>
+        <v>32.85</v>
       </c>
       <c r="O28" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: R$ 20,62 7 dias úteis PAC R$ 26,55 5 dias úteis Jadlog Package R$ 40,39 3 dias úteis SEDEX</t>
+          <t>Opção mais barata para o CEP 74933-130: Pac R$ 32,85 De 9 A 10 dia(s) Úteis</t>
         </is>
       </c>
       <c r="P28" s="2" t="n"/>
@@ -2271,7 +2269,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="E29" s="4" t="n">
@@ -2279,38 +2277,38 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>LOJAS 360 INDUSTRIA, COMERCIO, IMPORTACAO, EXPORTACAO LTDA</t>
+          <t>BHZ EPI DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>27.061.442/0002-85</t>
+          <t>31.893.116/0001-20</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr">
         <is>
-          <t>https://www.lojas360.com.br/protecao-das-maos/luva-latex-neoprene-amareloazul-pl-7004-plastcor-c-a-43916?variant_id=5131</t>
+          <t>https://www.loja.bhzepi.com.br/luva-latex-neoprene-bicolor-ca16779-volk</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Luva Látex Neoprene Amarelo/Azul Pl 7004 Plastcor | C.A. 43916</t>
+          <t>LUVA LATEX NEOPRENE BICOLOR CA16779 VOLK (Tamanho: M)</t>
         </is>
       </c>
       <c r="J29" s="6" t="n">
-        <v>9.31</v>
+        <v>13</v>
       </c>
       <c r="K29" s="2" t="n"/>
       <c r="L29" s="2" t="n"/>
       <c r="M29" s="6" t="n">
-        <v>9.31</v>
+        <v>13</v>
       </c>
       <c r="N29" s="6" t="n">
-        <v>18.4</v>
+        <v>20.62</v>
       </c>
       <c r="O29" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: SEDEX R$ 28,85 Até 6 dias úteis após o faturamento do pedido.rn PAC R$ 18,40 Até 10 dias úteis após o faturamento do pedido.rn Logística Própria FAVOR</t>
+          <t>Opção mais barata para o CEP 74933-130: R$ 20,62 7 dias úteis PAC R$ 26,55 5 dias úteis Jadlog Package R$ 40,39 3 dias úteis SEDEX</t>
         </is>
       </c>
       <c r="P29" s="2" t="n"/>
@@ -2341,38 +2339,38 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>SEGURANCA TOTAL EPIS LTDA</t>
+          <t>LOJAS 360 INDUSTRIA, COMERCIO, IMPORTACAO, EXPORTACAO LTDA</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>39.268.527/0001-37</t>
+          <t>27.061.442/0002-85</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>https://www.segurancatotal.com.br/luva-latexneoprene-supermix-super-safety-ca-33333</t>
+          <t>https://www.lojas360.com.br/protecao-das-maos/luva-latex-neoprene-amareloazul-pl-7004-plastcor-c-a-43916?variant_id=5131</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Luva Látex/Neoprene Supermix Super Safety CA 33333 (Tamanho das Luvas: 7/P)</t>
+          <t>Luva Látex Neoprene Amarelo/Azul Pl 7004 Plastcor | C.A. 43916</t>
         </is>
       </c>
       <c r="J30" s="6" t="n">
-        <v>10.41</v>
+        <v>9.31</v>
       </c>
       <c r="K30" s="2" t="n"/>
       <c r="L30" s="2" t="n"/>
       <c r="M30" s="6" t="n">
-        <v>10.41</v>
+        <v>9.31</v>
       </c>
       <c r="N30" s="6" t="n">
         <v>18.4</v>
       </c>
       <c r="O30" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: R$ 18,40 7 dias úteis PAC R$ 28,85 3 dias úteis SEDEX</t>
+          <t>Opção mais barata para o CEP 74933-130: SEDEX R$ 28,85 Até 6 dias úteis após o faturamento do pedido.rn PAC R$ 18,40 Até 10 dias úteis após o faturamento do pedido.rn Logística Própria FAVOR</t>
         </is>
       </c>
       <c r="P30" s="2" t="n"/>
@@ -2395,44 +2393,46 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E31" s="4" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Goiás Ferramentas</t>
+          <t>SEGURANCA TOTAL EPIS LTDA</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>09.497.806/0001-01</t>
+          <t>39.268.527/0001-37</t>
         </is>
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>https://www.goiasferramentas.com.br/produto/13963-luva-de-latex-neoprene-kalipso-neoprex-azul-e-amarela-xg</t>
+          <t>https://www.segurancatotal.com.br/luva-latexneoprene-supermix-super-safety-ca-33333</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>Luva de Latex / Neoprene Kalipso Neoprex Azul e Amarela XG</t>
+          <t>Luva Látex/Neoprene Supermix Super Safety CA 33333 (Tamanho das Luvas: 7/P)</t>
         </is>
       </c>
       <c r="J31" s="6" t="n">
-        <v>10.88</v>
+        <v>10.41</v>
       </c>
       <c r="K31" s="2" t="n"/>
       <c r="L31" s="2" t="n"/>
       <c r="M31" s="6" t="n">
-        <v>10.88</v>
-      </c>
-      <c r="N31" s="2" t="n"/>
+        <v>10.41</v>
+      </c>
+      <c r="N31" s="6" t="n">
+        <v>18.4</v>
+      </c>
       <c r="O31" s="3" t="inlineStr">
         <is>
-          <t>Frete não calculado (GO para GO)</t>
+          <t>Opção mais barata para o CEP 74933-130: R$ 18,40 7 dias úteis PAC R$ 28,85 3 dias úteis SEDEX</t>
         </is>
       </c>
       <c r="P31" s="2" t="n"/>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="E32" s="4" t="n">
@@ -2463,38 +2463,36 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>A Master EPI</t>
+          <t>Goiás Ferramentas</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>16.603.654/0001-40</t>
+          <t>09.497.806/0001-01</t>
         </is>
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>https://www.amasterepi.com.br/21946/luva-de-latex-neoprene-bicolor-std-volk-p</t>
+          <t>https://www.goiasferramentas.com.br/produto/13963-luva-de-latex-neoprene-kalipso-neoprex-azul-e-amarela-xg</t>
         </is>
       </c>
       <c r="I32" s="3" t="inlineStr">
         <is>
-          <t>Luva de Latex Neoprene Bicolor Std Volk</t>
+          <t>Luva de Latex / Neoprene Kalipso Neoprex Azul e Amarela XG</t>
         </is>
       </c>
       <c r="J32" s="6" t="n">
-        <v>10.5</v>
+        <v>10.88</v>
       </c>
       <c r="K32" s="2" t="n"/>
       <c r="L32" s="2" t="n"/>
       <c r="M32" s="6" t="n">
-        <v>10.5</v>
-      </c>
-      <c r="N32" s="6" t="n">
-        <v>32.85</v>
-      </c>
+        <v>10.88</v>
+      </c>
+      <c r="N32" s="2" t="n"/>
       <c r="O32" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: Entrega Econômica R$ 32,85 De 6 A 7 dia(s) Úteis</t>
+          <t>Frete não calculado (GO para GO)</t>
         </is>
       </c>
       <c r="P32" s="2" t="n"/>
@@ -2507,56 +2505,56 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>1112</t>
+          <t>1111</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>LUVA DE ALGODÃO PIGMENTADA - PARA ATIVIDADES DE APOIO/MANUSEIO.</t>
+          <t>LUVA DE NEOPRENE - TAMANHOS VARIADOS; PARA MANIPULAÇÃO COMPATÍVEL DE PRODUTOS QUÍMICOS.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>PR</t>
         </is>
       </c>
       <c r="E33" s="4" t="n">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>SEGURANCA TOTAL EPIS LTDA</t>
+          <t>A Master EPI</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>39.268.527/0001-37</t>
+          <t>16.603.654/0001-40</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>https://www.segurancatotal.com.br/produto/luva-tricotada-pigmentada-preta-handex-4-fios.html</t>
+          <t>https://www.amasterepi.com.br/21946/luva-de-latex-neoprene-bicolor-std-volk-p</t>
         </is>
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>Luva Tricotada Pigmentada Preta Handex 4 Fios</t>
+          <t>Luva de Latex Neoprene Bicolor Std Volk</t>
         </is>
       </c>
       <c r="J33" s="6" t="n">
-        <v>3.09</v>
+        <v>10.5</v>
       </c>
       <c r="K33" s="2" t="n"/>
       <c r="L33" s="2" t="n"/>
       <c r="M33" s="6" t="n">
-        <v>3.09</v>
+        <v>10.5</v>
       </c>
       <c r="N33" s="6" t="n">
-        <v>18.4</v>
+        <v>32.85</v>
       </c>
       <c r="O33" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: R$ 18,40 7 dias úteis PAC R$ 28,85 3 dias úteis SEDEX</t>
+          <t>Opção mais barata para o CEP 74933-130: Entrega Econômica R$ 32,85 De 6 A 7 dia(s) Úteis</t>
         </is>
       </c>
       <c r="P33" s="2" t="n"/>
@@ -2579,46 +2577,46 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>PR</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E34" s="4" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>TR Distribuidora</t>
+          <t>SEGURANCA TOTAL EPIS LTDA</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>14.213.841/0001-91</t>
+          <t>39.268.527/0001-37</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>https://www.trepis.com.br/luva-em-algodao-tricotada-modelo-cotton-black-sem-banho-e-com-pigmento-riscos-mecanicos-c-a-36347</t>
+          <t>https://www.segurancatotal.com.br/produto/luva-tricotada-pigmentada-preta-handex-4-fios.html</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
-          <t>Luva de Algodão Tricotada Cotton Black Pigmentada para Riscos Mecânicos C.A. 36347</t>
+          <t>Luva Tricotada Pigmentada Preta Handex 4 Fios</t>
         </is>
       </c>
       <c r="J34" s="6" t="n">
-        <v>2.82</v>
+        <v>3.09</v>
       </c>
       <c r="K34" s="2" t="n"/>
       <c r="L34" s="2" t="n"/>
       <c r="M34" s="6" t="n">
-        <v>2.82</v>
+        <v>3.09</v>
       </c>
       <c r="N34" s="6" t="n">
-        <v>21.55</v>
+        <v>18.4</v>
       </c>
       <c r="O34" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: JADLOG .Package R$ 21,55 Capital de todo Brasil: 01 a 03 dias. Interior de Todo Brasil: 02 a 05 dias.</t>
+          <t>Opção mais barata para o CEP 74933-130: R$ 18,40 7 dias úteis PAC R$ 28,85 3 dias úteis SEDEX</t>
         </is>
       </c>
       <c r="P34" s="2" t="n"/>
@@ -2641,48 +2639,46 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>MG</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>14/10/2026</t>
-        </is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>46304</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>BHZ EPI DISTRIBUIDORA LTDA</t>
+          <t>TR Distribuidora</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>31.893.116/0001-20</t>
+          <t>14.213.841/0001-91</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>https://www.loja.bhzepi.com.br/luva-de-segurana-malha-tricotada-pigmentada-branca</t>
+          <t>https://www.trepis.com.br/luva-em-algodao-tricotada-modelo-cotton-black-sem-banho-e-com-pigmento-riscos-mecanicos-c-a-36347</t>
         </is>
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>Luva De Segurança Malha Tricotada Pigmentada branca</t>
+          <t>Luva de Algodão Tricotada Cotton Black Pigmentada para Riscos Mecânicos C.A. 36347</t>
         </is>
       </c>
       <c r="J35" s="6" t="n">
-        <v>3.9</v>
+        <v>2.82</v>
       </c>
       <c r="K35" s="2" t="n"/>
       <c r="L35" s="2" t="n"/>
       <c r="M35" s="6" t="n">
-        <v>3.9</v>
+        <v>2.82</v>
       </c>
       <c r="N35" s="6" t="n">
-        <v>20.62</v>
+        <v>21.55</v>
       </c>
       <c r="O35" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: R$ 20,62 7 dias úteis PAC</t>
+          <t>Opção mais barata para o CEP 74933-130: JADLOG .Package R$ 21,55 Capital de todo Brasil: 01 a 03 dias. Interior de Todo Brasil: 02 a 05 dias.</t>
         </is>
       </c>
       <c r="P35" s="2" t="n"/>
@@ -2705,46 +2701,48 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="n">
-        <v>46308</v>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>Dimensional Brasil Solucoes Ltda</t>
+          <t>BHZ EPI DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>06.913.480/0001-68</t>
+          <t>31.893.116/0001-20</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>https://www.dimensional.com.br/luva-algodaopoliester-preta-pigmentada-tamanho-9-tatex-021123-kalipso/p</t>
+          <t>https://www.loja.bhzepi.com.br/luva-de-segurana-malha-tricotada-pigmentada-branca</t>
         </is>
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>Luva Algodao/Poliester Preta Pigmentada Tatex 02.11.2.3 Tamanho 9 Kalipso</t>
+          <t>Luva De Segurança Malha Tricotada Pigmentada branca</t>
         </is>
       </c>
       <c r="J36" s="6" t="n">
-        <v>2.09</v>
+        <v>3.9</v>
       </c>
       <c r="K36" s="2" t="n"/>
       <c r="L36" s="2" t="n"/>
       <c r="M36" s="6" t="n">
-        <v>2.09</v>
+        <v>3.9</v>
       </c>
       <c r="N36" s="6" t="n">
-        <v>52.84</v>
+        <v>20.62</v>
       </c>
       <c r="O36" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: Transportadora Em até 6 dias úteis R$ 52,84</t>
+          <t>Opção mais barata para o CEP 74933-130: R$ 20,62 7 dias úteis PAC</t>
         </is>
       </c>
       <c r="P36" s="2" t="n"/>
@@ -2757,17 +2755,17 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>1113</t>
+          <t>1112</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>ÓCULOS DE PROTEÇÃO INCOLOR - PARA MANIPULAÇÃO E APLICAÇÃO DE PRODUTOS QUÍMICOS.</t>
+          <t>LUVA DE ALGODÃO PIGMENTADA - PARA ATIVIDADES DE APOIO/MANUSEIO.</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>MG</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E37" s="4" t="n">
@@ -2775,38 +2773,38 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>BHZ EPI DISTRIBUIDORA LTDA</t>
+          <t>Dimensional Brasil Solucoes Ltda</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>31.893.116/0001-20</t>
+          <t>06.913.480/0001-68</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">
         <is>
-          <t>https://www.loja.bhzepi.com.br/produto/oculos-de-seguranca-roma-incolor-protecao-uv-antirrisco</t>
+          <t>https://www.dimensional.com.br/luva-algodaopoliester-preta-pigmentada-tamanho-9-tatex-021123-kalipso/p</t>
         </is>
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>Oculos De Segurança Roma Incolor Proteção Uv Antirrisco</t>
+          <t>Luva Algodao/Poliester Preta Pigmentada Tatex 02.11.2.3 Tamanho 9 Kalipso</t>
         </is>
       </c>
       <c r="J37" s="6" t="n">
-        <v>70</v>
+        <v>2.09</v>
       </c>
       <c r="K37" s="2" t="n"/>
       <c r="L37" s="2" t="n"/>
       <c r="M37" s="6" t="n">
-        <v>70</v>
+        <v>2.09</v>
       </c>
       <c r="N37" s="6" t="n">
-        <v>20.62</v>
+        <v>52.84</v>
       </c>
       <c r="O37" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: R$ 20,62 7 dias úteis PAC R$ 26,55 5 dias úteis Jadlog Package R$ 40,39 3 dias úteis SEDEX</t>
+          <t>Opção mais barata para o CEP 74933-130: Transportadora Em até 6 dias úteis R$ 52,84</t>
         </is>
       </c>
       <c r="P37" s="2" t="n"/>
@@ -2829,7 +2827,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
+          <t>MG</t>
         </is>
       </c>
       <c r="E38" s="4" t="n">
@@ -2837,38 +2835,38 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>LOJAS 360 INDUSTRIA, COMERCIO, IMPORTACAO, EXPORTACAO LTDA</t>
+          <t>BHZ EPI DISTRIBUIDORA LTDA</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>27.061.442/0002-85</t>
+          <t>31.893.116/0001-20</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>https://www.lojas360.com.br/oculos-de-seguranca-urano</t>
+          <t>https://www.loja.bhzepi.com.br/produto/oculos-de-seguranca-roma-incolor-protecao-uv-antirrisco</t>
         </is>
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>Óculos de Segurança Urano Incolor Anti Risco | C.A. 42547</t>
+          <t>Oculos De Segurança Roma Incolor Proteção Uv Antirrisco</t>
         </is>
       </c>
       <c r="J38" s="6" t="n">
-        <v>9.41</v>
+        <v>70</v>
       </c>
       <c r="K38" s="2" t="n"/>
       <c r="L38" s="2" t="n"/>
       <c r="M38" s="6" t="n">
-        <v>9.41</v>
+        <v>70</v>
       </c>
       <c r="N38" s="6" t="n">
-        <v>18.4</v>
+        <v>20.62</v>
       </c>
       <c r="O38" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: SEDEX R$ 28,85 Até 6 dias úteis após o faturamento do pedido.rn PAC R$ 18,40 Até 10 dias úteis após o faturamento do pedido.rn Logística Própria FAVOR</t>
+          <t>Opção mais barata para o CEP 74933-130: R$ 20,62 7 dias úteis PAC R$ 26,55 5 dias úteis Jadlog Package R$ 40,39 3 dias úteis SEDEX</t>
         </is>
       </c>
       <c r="P38" s="2" t="n"/>
@@ -2899,38 +2897,38 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>SEGURANCA TOTAL EPIS LTDA</t>
+          <t>LOJAS 360 INDUSTRIA, COMERCIO, IMPORTACAO, EXPORTACAO LTDA</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>39.268.527/0001-37</t>
+          <t>27.061.442/0002-85</t>
         </is>
       </c>
       <c r="H39" s="5" t="inlineStr">
         <is>
-          <t>https://www.segurancatotal.com.br/produto/oculos-de-protecao-sky-deltaplus-incolor.html</t>
+          <t>https://www.lojas360.com.br/oculos-de-seguranca-urano</t>
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr">
         <is>
-          <t>Óculos De Proteção Sky Deltaplus Incolor</t>
+          <t>Óculos de Segurança Urano Incolor Anti Risco | C.A. 42547</t>
         </is>
       </c>
       <c r="J39" s="6" t="n">
-        <v>3.99</v>
+        <v>9.41</v>
       </c>
       <c r="K39" s="2" t="n"/>
       <c r="L39" s="2" t="n"/>
       <c r="M39" s="6" t="n">
-        <v>3.99</v>
+        <v>9.41</v>
       </c>
       <c r="N39" s="6" t="n">
         <v>18.4</v>
       </c>
       <c r="O39" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: R$ 18,40 7 dias úteis PAC R$ 28,85 3 dias úteis SEDEX</t>
+          <t>Opção mais barata para o CEP 74933-130: SEDEX R$ 28,85 Até 6 dias úteis após o faturamento do pedido.rn PAC R$ 18,40 Até 10 dias úteis após o faturamento do pedido.rn Logística Própria FAVOR</t>
         </is>
       </c>
       <c r="P39" s="2" t="n"/>
@@ -2953,7 +2951,7 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>SP</t>
         </is>
       </c>
       <c r="E40" s="4" t="n">
@@ -2961,36 +2959,38 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>ZEUS DO BRASIL LTDA (loja EPI Zeus)</t>
+          <t>SEGURANCA TOTAL EPIS LTDA</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>82.699.588/0001-88</t>
+          <t>39.268.527/0001-37</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>https://www.epizeus.com.br/oculos-protec-o-lente-incolor-policarbonato-ca-28018</t>
+          <t>https://www.segurancatotal.com.br/produto/oculos-de-protecao-sky-deltaplus-incolor.html</t>
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr">
         <is>
-          <t>Óculos proteção lente incolor policarbonato - CA 10346</t>
+          <t>Óculos De Proteção Sky Deltaplus Incolor</t>
         </is>
       </c>
       <c r="J40" s="6" t="n">
-        <v>15.9</v>
+        <v>3.99</v>
       </c>
       <c r="K40" s="2" t="n"/>
       <c r="L40" s="2" t="n"/>
       <c r="M40" s="6" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="N40" s="2" t="n"/>
+        <v>3.99</v>
+      </c>
+      <c r="N40" s="6" t="n">
+        <v>18.4</v>
+      </c>
       <c r="O40" s="3" t="inlineStr">
         <is>
-          <t>Frete grátis informado na página do produto: "🚚 FRETE GRÁTIS PARA TODO O BRASIL*" (sem calculadora de CEP no site)</t>
+          <t>Opção mais barata para o CEP 74933-130: R$ 18,40 7 dias úteis PAC R$ 28,85 3 dias úteis SEDEX</t>
         </is>
       </c>
       <c r="P40" s="2" t="n"/>
@@ -3013,48 +3013,44 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>SP</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>14/10/2026</t>
-        </is>
+          <t>SC</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>46308</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>SINGULAR COMERCIO DE EQUIPAMENTOS DE PROTECAO INDIVIDUAL LTDA (Loja do EPI)</t>
+          <t>ZEUS DO BRASIL LTDA (loja EPI Zeus)</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>20.838.307/0001-73</t>
+          <t>82.699.588/0001-88</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr">
         <is>
-          <t>https://www.lojadoepi.com.br/oculos-de-protecao-vvision-600-incolor-antiembacante-volk-ca-42922-p3187</t>
+          <t>https://www.epizeus.com.br/oculos-protec-o-lente-incolor-policarbonato-ca-28018</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Óculos de Proteção Vvision 600 Incolor Antiembaçante Volk CA 42922</t>
+          <t>Óculos proteção lente incolor policarbonato - CA 10346</t>
         </is>
       </c>
       <c r="J41" s="6" t="n">
-        <v>26.93</v>
+        <v>15.9</v>
       </c>
       <c r="K41" s="2" t="n"/>
       <c r="L41" s="2" t="n"/>
       <c r="M41" s="6" t="n">
-        <v>26.93</v>
-      </c>
-      <c r="N41" s="6" t="n">
-        <v>21.39</v>
-      </c>
+        <v>15.9</v>
+      </c>
+      <c r="N41" s="2" t="n"/>
       <c r="O41" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: Pac R$ 21,39 7 dia(s) útil(eis)</t>
+          <t>Frete grátis informado na página do produto: "🚚 FRETE GRÁTIS PARA TODO O BRASIL*" (sem calculadora de CEP no site)</t>
         </is>
       </c>
       <c r="P41" s="2" t="n"/>
@@ -3077,43 +3073,47 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>RS</t>
+          <t>GO</t>
         </is>
       </c>
       <c r="E42" s="4" t="n">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>SUPRIFLEX SUPRIMENTOS ONLINE LTDA</t>
+          <t>Casa do Pica-Pau</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>46.412.993/0001-00</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="n"/>
+          <t>50.223.823/0001-54</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>https://www.casadopicapau.com.br/oculos-de-protecao-stihl-policarbonato-incolor/p?skuId=5055</t>
+        </is>
+      </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>ÓCULOS SEGURANCA DISMA II INCOLOR</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="n"/>
+          <t>Óculos de Proteção STIHL em Policarbonato Incolor</t>
+        </is>
+      </c>
+      <c r="J42" s="6" t="n">
+        <v>16.1</v>
+      </c>
       <c r="K42" s="2" t="n"/>
       <c r="L42" s="2" t="n"/>
-      <c r="M42" s="2" t="n"/>
+      <c r="M42" s="6" t="n">
+        <v>16.1</v>
+      </c>
       <c r="N42" s="2" t="n"/>
       <c r="O42" s="3" t="inlineStr">
         <is>
-          <t>Preço não exibido (motivo não identificado)</t>
-        </is>
-      </c>
-      <c r="P42" s="5" t="inlineStr">
-        <is>
-          <t>https://www.supriflex.com.br/produto/oculos-seguranca-disma-ii-incolor.html</t>
-        </is>
-      </c>
+          <t>Frete não calculado (GO para GO)</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3123,17 +3123,17 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>1114</t>
+          <t>1113</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>MÁSCARA DE PROTEÇÃO DESCARTÁVEL - USO CONFORME RISCO/ATIVIDADE.</t>
+          <t>ÓCULOS DE PROTEÇÃO INCOLOR - PARA MANIPULAÇÃO E APLICAÇÃO DE PRODUTOS QUÍMICOS.</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
+          <t>RS</t>
         </is>
       </c>
       <c r="E43" s="4" t="n">
@@ -3141,39 +3141,35 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>ZEUS DO BRASIL LTDA (loja EPI Zeus)</t>
+          <t>SUPRIFLEX SUPRIMENTOS ONLINE LTDA</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>82.699.588/0001-88</t>
-        </is>
-      </c>
-      <c r="H43" s="5" t="inlineStr">
-        <is>
-          <t>https://www.epizeus.com.br/mascara-de-protec-o-pff1-sem-valvula-delta-plus-ca-38502</t>
-        </is>
-      </c>
+          <t>46.412.993/0001-00</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="n"/>
       <c r="I43" s="3" t="inlineStr">
         <is>
-          <t>Máscara de Proteção PFF1 - Sem Válvula - CA 45020</t>
-        </is>
-      </c>
-      <c r="J43" s="6" t="n">
-        <v>1.9</v>
-      </c>
+          <t>ÓCULOS SEGURANCA DISMA II INCOLOR</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="n"/>
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="n"/>
-      <c r="M43" s="6" t="n">
-        <v>1.9</v>
-      </c>
+      <c r="M43" s="2" t="n"/>
       <c r="N43" s="2" t="n"/>
       <c r="O43" s="3" t="inlineStr">
         <is>
-          <t>Frete grátis informado na página do produto: "🚚 FRETE GRÁTIS PARA TODO O BRASIL*" (sem calculadora de CEP no site)</t>
-        </is>
-      </c>
-      <c r="P43" s="2" t="n"/>
+          <t>Preço não exibido (motivo não identificado)</t>
+        </is>
+      </c>
+      <c r="P43" s="5" t="inlineStr">
+        <is>
+          <t>https://www.supriflex.com.br/produto/oculos-seguranca-disma-ii-incolor.html</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3193,30 +3189,30 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>SC</t>
         </is>
       </c>
       <c r="E44" s="4" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>Goiás Ferramentas</t>
+          <t>ZEUS DO BRASIL LTDA (loja EPI Zeus)</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>09.497.806/0001-01</t>
+          <t>82.699.588/0001-88</t>
         </is>
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>https://www.goiasferramentas.com.br/produto/10985-mascara-descartavel-pff2-com-valvula</t>
+          <t>https://www.epizeus.com.br/mascara-de-protec-o-pff1-sem-valvula-delta-plus-ca-38502</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>MASCARA DESCARTAVEL PFF2 COM VALVULA</t>
+          <t>Máscara de Proteção PFF1 - Sem Válvula - CA 45020</t>
         </is>
       </c>
       <c r="J44" s="6" t="n">
@@ -3230,7 +3226,7 @@
       <c r="N44" s="2" t="n"/>
       <c r="O44" s="3" t="inlineStr">
         <is>
-          <t>Frete não calculado (GO para GO)</t>
+          <t>Frete grátis informado na página do produto: "🚚 FRETE GRÁTIS PARA TODO O BRASIL*" (sem calculadora de CEP no site)</t>
         </is>
       </c>
       <c r="P44" s="2" t="n"/>
@@ -3257,39 +3253,35 @@
         </is>
       </c>
       <c r="E45" s="4" t="n">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>Fermarcs Ferramentas</t>
+          <t>Mais Segurança EPI</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>08.615.223/0001-75</t>
+          <t>43.903.641/0001-69</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>https://www.fermarcsferramentas.com.br/epi-e-epc/respiratoria/mascara-de-protecao-msk95-pff-2-n95</t>
+          <t>https://maisseguranca.online/#/produto-detalhes/nUNEWOBUivWtuxf5g7uS3ulpNCn2/-NWsT-o_-VgTH2z0Xn2v</t>
         </is>
       </c>
       <c r="I45" s="3" t="inlineStr">
         <is>
-          <t>Mascara De Protecao Msk95 Pff-2 N95</t>
+          <t>RESPIRADOR PFF2 AZ S/VALV PRO SAFETY - DELTA PLUS CA.38504</t>
         </is>
       </c>
       <c r="J45" s="6" t="n">
-        <v>2.99</v>
+        <v>1</v>
       </c>
       <c r="K45" s="2" t="n"/>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>Característica não confirmada na página do produto: descartável.</t>
-        </is>
-      </c>
+      <c r="L45" s="2" t="n"/>
       <c r="M45" s="6" t="n">
-        <v>2.99</v>
+        <v>1</v>
       </c>
       <c r="N45" s="2" t="n"/>
       <c r="O45" s="3" t="inlineStr">
@@ -3317,48 +3309,44 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>PR</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>14/10/2026</t>
-        </is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>46307</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>TR Distribuidora de Equipamentos de Segurança LTDA</t>
+          <t>Goiás Ferramentas</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>14.213.841/0001-91</t>
+          <t>09.497.806/0001-01</t>
         </is>
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>https://www.trepis.com.br/mascara-descartavel-confec-em-tnt-tripla-branca-com-elastico-pct-c50un</t>
+          <t>https://www.goiasferramentas.com.br/produto/10985-mascara-descartavel-pff2-com-valvula</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Máscara Descartável Tripla TNT Branca com Elástico Pacote com 50 Unidades</t>
+          <t>MASCARA DESCARTAVEL PFF2 COM VALVULA</t>
         </is>
       </c>
       <c r="J46" s="6" t="n">
-        <v>10.81</v>
+        <v>1.9</v>
       </c>
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="n"/>
       <c r="M46" s="6" t="n">
-        <v>10.81</v>
-      </c>
-      <c r="N46" s="6" t="n">
-        <v>21.55</v>
-      </c>
+        <v>1.9</v>
+      </c>
+      <c r="N46" s="2" t="n"/>
       <c r="O46" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: JADLOG .Package R$ 21,55 Capital de todo Brasil: 01 a 03 dias. Interior de Todo Brasil: 02 a 05 dias.</t>
+          <t>Frete não calculado (GO para GO)</t>
         </is>
       </c>
       <c r="P46" s="2" t="n"/>
@@ -3381,48 +3369,48 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>SC</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>14/10/2026</t>
-        </is>
+          <t>GO</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>46307</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>ASTRO DISTRIBUIDORA LTDA</t>
+          <t>Fermarcs Ferramentas</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>18.597.685/0001-60</t>
+          <t>08.615.223/0001-75</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>https://www.astrodistribuidora.com/mascara-de-tnt-descartavel-com-elastico-volk</t>
+          <t>https://www.fermarcsferramentas.com.br/epi-e-epc/respiratoria/mascara-de-protecao-msk95-pff-2-n95</t>
         </is>
       </c>
       <c r="I47" s="3" t="inlineStr">
         <is>
-          <t>Máscara de TNT Descartável com Elástico - Volk (100 Unidades)</t>
+          <t>Mascara De Protecao Msk95 Pff-2 N95</t>
         </is>
       </c>
       <c r="J47" s="6" t="n">
-        <v>10.42</v>
+        <v>2.99</v>
       </c>
       <c r="K47" s="2" t="n"/>
-      <c r="L47" s="2" t="n"/>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>Característica não confirmada na página do produto: descartável.</t>
+        </is>
+      </c>
       <c r="M47" s="6" t="n">
-        <v>10.42</v>
-      </c>
-      <c r="N47" s="6" t="n">
-        <v>26.82</v>
-      </c>
+        <v>2.99</v>
+      </c>
+      <c r="N47" s="2" t="n"/>
       <c r="O47" s="3" t="inlineStr">
         <is>
-          <t>Opção mais barata para o CEP 74933-130: JADLOG - Entrega em até 5 dias úteis - R$26,82 BRASPRESS - Entrega em até 15 dias úteis -</t>
+          <t>Frete não calculado (GO para GO)</t>
         </is>
       </c>
       <c r="P47" s="2" t="n"/>
@@ -5251,8 +5239,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P14" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId16"/>
@@ -5280,8 +5268,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H39" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H40" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H41" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P42" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H44" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H45" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H46" r:id="rId45"/>

</xml_diff>